<commit_message>
Snapshot History Test Cases
</commit_message>
<xml_diff>
--- a/src/main/resources/Program_Field_Values_QA_org.xlsx
+++ b/src/main/resources/Program_Field_Values_QA_org.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25601"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25831"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F57C38F-5878-4036-B4D9-596892C4C048}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11DDE804-503E-4F67-B0F9-3044EAC38D31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="6" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ProgramCreation_v" sheetId="22" r:id="rId1"/>
@@ -869,6 +869,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1534,7 +1535,7 @@
         <v>63</v>
       </c>
       <c r="C3">
-        <v>730</v>
+        <v>1825</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -1619,6 +1620,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Rename feature file and Automate E-Grid test cases
</commit_message>
<xml_diff>
--- a/src/main/resources/Program_Field_Values_QA_org.xlsx
+++ b/src/main/resources/Program_Field_Values_QA_org.xlsx
@@ -3,26 +3,27 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25831"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11DDE804-503E-4F67-B0F9-3044EAC38D31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F91ACA1-67DA-4554-BB73-FC4EAC94C9E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ProgramCreation_v" sheetId="22" r:id="rId1"/>
     <sheet name="ProgramEdition_v" sheetId="23" r:id="rId2"/>
-    <sheet name="NewOrgAnnCreation_v" sheetId="24" r:id="rId3"/>
-    <sheet name="NewOrg2ndModal_v" sheetId="25" r:id="rId4"/>
-    <sheet name="NewOrgAnnEdition_v" sheetId="26" r:id="rId5"/>
-    <sheet name="NewOrgAppEddition_v" sheetId="27" r:id="rId6"/>
-    <sheet name="StandardAssurancesForm_v" sheetId="28" r:id="rId7"/>
-    <sheet name="ProgramApplicationForm_v" sheetId="29" r:id="rId8"/>
-    <sheet name="PaymentRequestSchedule_v" sheetId="30" r:id="rId9"/>
-    <sheet name="GrantCreation_v" sheetId="31" r:id="rId10"/>
-    <sheet name="Grant_Edition_v" sheetId="32" r:id="rId11"/>
-    <sheet name="StandAloneEdition_v" sheetId="33" r:id="rId12"/>
-    <sheet name="SiteVisitCreation_v" sheetId="34" r:id="rId13"/>
-    <sheet name="SiteVisitEdition_v" sheetId="35" r:id="rId14"/>
-    <sheet name="GeneralReviewForm_v" sheetId="36" r:id="rId15"/>
+    <sheet name="ProgramEditon_forCkEditor" sheetId="37" r:id="rId3"/>
+    <sheet name="NewOrgAnnCreation_v" sheetId="24" r:id="rId4"/>
+    <sheet name="NewOrg2ndModal_v" sheetId="25" r:id="rId5"/>
+    <sheet name="NewOrgAnnEdition_v" sheetId="26" r:id="rId6"/>
+    <sheet name="NewOrgAppEddition_v" sheetId="27" r:id="rId7"/>
+    <sheet name="StandardAssurancesForm_v" sheetId="28" r:id="rId8"/>
+    <sheet name="ProgramApplicationForm_v" sheetId="29" r:id="rId9"/>
+    <sheet name="PaymentRequestSchedule_v" sheetId="30" r:id="rId10"/>
+    <sheet name="GrantCreation_v" sheetId="31" r:id="rId11"/>
+    <sheet name="Grant_Edition_v" sheetId="32" r:id="rId12"/>
+    <sheet name="StandAloneEdition_v" sheetId="33" r:id="rId13"/>
+    <sheet name="SiteVisitCreation_v" sheetId="34" r:id="rId14"/>
+    <sheet name="SiteVisitEdition_v" sheetId="35" r:id="rId15"/>
+    <sheet name="GeneralReviewForm_v" sheetId="36" r:id="rId16"/>
   </sheets>
   <calcPr calcId="179017"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="132">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -784,13 +785,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E83D430-2DDF-4C96-A733-8F6A18593E6C}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="30.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -801,7 +802,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -812,7 +813,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -823,7 +824,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -834,7 +835,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -845,7 +846,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -856,7 +857,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -874,111 +875,56 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8CB8E10-5A8B-4AF3-AF66-F1E9AA7C9BBC}">
-  <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B88D2545-36F8-47CF-B9C1-1EF7F48C6F22}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="27.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="33.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="4" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B2" t="s">
+        <v>101</v>
+      </c>
+      <c r="C2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="6" t="s">
-        <v>104</v>
+      <c r="B3" t="s">
+        <v>102</v>
       </c>
       <c r="C3" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="6" t="s">
-        <v>105</v>
-      </c>
-      <c r="C4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>106</v>
-      </c>
-      <c r="C5">
-        <v>365</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>107</v>
-      </c>
-      <c r="C6" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="C7" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="C8" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>109</v>
-      </c>
-      <c r="C9" t="s">
-        <v>131</v>
+      <c r="B4" t="s">
+        <v>103</v>
+      </c>
+      <c r="C4" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -987,15 +933,15 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55BEB37B-B28E-4F60-BECB-CD35E74B4C36}">
-  <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8CB8E10-5A8B-4AF3-AF66-F1E9AA7C9BBC}">
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="27.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1006,125 +952,92 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B2" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
-      <c r="B3" t="s">
-        <v>12</v>
+      <c r="B3" s="6" t="s">
+        <v>104</v>
       </c>
       <c r="C3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B4" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>3</v>
       </c>
-      <c r="B5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B5" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="C5">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>3</v>
       </c>
-      <c r="B6" t="s">
-        <v>49</v>
+      <c r="B6" s="6" t="s">
+        <v>107</v>
       </c>
       <c r="C6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>3</v>
       </c>
-      <c r="B7" t="s">
-        <v>8</v>
+      <c r="B7" s="6" t="s">
+        <v>48</v>
       </c>
       <c r="C7" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>3</v>
       </c>
-      <c r="B8" t="s">
-        <v>7</v>
+      <c r="B8" s="6" t="s">
+        <v>70</v>
       </c>
       <c r="C8" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>3</v>
       </c>
-      <c r="B9" t="s">
-        <v>15</v>
+      <c r="B9" s="6" t="s">
+        <v>109</v>
       </c>
       <c r="C9" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" t="s">
-        <v>50</v>
-      </c>
-      <c r="C10" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" t="s">
-        <v>14</v>
-      </c>
-      <c r="C11" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>3</v>
-      </c>
-      <c r="B12" t="s">
-        <v>66</v>
-      </c>
-      <c r="C12" t="s">
-        <v>9</v>
+        <v>131</v>
       </c>
     </row>
   </sheetData>
@@ -1133,15 +1046,15 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82865F4C-F847-4F90-8B11-C831BFCC23C2}">
-  <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55BEB37B-B28E-4F60-BECB-CD35E74B4C36}">
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="30" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1152,59 +1065,125 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>110</v>
+        <v>11</v>
       </c>
       <c r="C2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>111</v>
+        <v>12</v>
       </c>
       <c r="C3" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>113</v>
+        <v>13</v>
       </c>
       <c r="C4" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>115</v>
-      </c>
-      <c r="C5">
-        <v>1234</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+        <v>16</v>
+      </c>
+      <c r="C5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>29</v>
+        <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>116</v>
-      </c>
-      <c r="C6">
-        <v>3650</v>
+        <v>49</v>
+      </c>
+      <c r="C6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
+        <v>50</v>
+      </c>
+      <c r="C10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" t="s">
+        <v>14</v>
+      </c>
+      <c r="C11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" t="s">
+        <v>66</v>
+      </c>
+      <c r="C12" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -1213,15 +1192,15 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDDAC24B-DC90-49E6-BD31-6F210026CA6D}">
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82865F4C-F847-4F90-8B11-C831BFCC23C2}">
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="25.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1232,37 +1211,59 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>117</v>
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>110</v>
       </c>
       <c r="C2" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>118</v>
+        <v>5</v>
+      </c>
+      <c r="B3" t="s">
+        <v>111</v>
       </c>
       <c r="C3" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>119</v>
+        <v>5</v>
+      </c>
+      <c r="B4" t="s">
+        <v>113</v>
       </c>
       <c r="C4" t="s">
-        <v>53</v>
+        <v>114</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" t="s">
+        <v>115</v>
+      </c>
+      <c r="C5">
+        <v>1234</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B6" t="s">
+        <v>116</v>
+      </c>
+      <c r="C6">
+        <v>3650</v>
       </c>
     </row>
   </sheetData>
@@ -1271,15 +1272,15 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6F7845C-214C-4C02-A5F4-6F38FB46E35D}">
-  <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDDAC24B-DC90-49E6-BD31-6F210026CA6D}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="33.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="41.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1290,81 +1291,37 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>120</v>
-      </c>
-      <c r="C2">
-        <v>365</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>3</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="C2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" t="s">
-        <v>121</v>
-      </c>
-      <c r="C3">
-        <v>455</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+        <v>3</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="C3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" t="s">
-        <v>54</v>
+        <v>3</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>119</v>
       </c>
       <c r="C4" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" t="s">
-        <v>56</v>
-      </c>
-      <c r="C5" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>5</v>
-      </c>
-      <c r="B6" t="s">
-        <v>57</v>
-      </c>
-      <c r="C6" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>5</v>
-      </c>
-      <c r="B7" t="s">
-        <v>59</v>
-      </c>
-      <c r="C7" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B8" t="s">
-        <v>61</v>
-      </c>
-      <c r="C8" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
   </sheetData>
@@ -1373,15 +1330,117 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6F7845C-214C-4C02-A5F4-6F38FB46E35D}">
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="33.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41.1796875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>120</v>
+      </c>
+      <c r="C2">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" t="s">
+        <v>121</v>
+      </c>
+      <c r="C3">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" t="s">
+        <v>54</v>
+      </c>
+      <c r="C4" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C5" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>57</v>
+      </c>
+      <c r="C6" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" t="s">
+        <v>59</v>
+      </c>
+      <c r="C7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" t="s">
+        <v>61</v>
+      </c>
+      <c r="C8" t="s">
+        <v>55</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE64D93B-66B6-48F6-99BC-E4BA23590E06}">
   <dimension ref="A1:C10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="23" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1392,7 +1451,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -1403,7 +1462,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -1414,7 +1473,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -1425,7 +1484,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -1436,7 +1495,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
@@ -1447,7 +1506,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>3</v>
       </c>
@@ -1458,7 +1517,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>3</v>
       </c>
@@ -1469,7 +1528,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>3</v>
       </c>
@@ -1480,7 +1539,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>3</v>
       </c>
@@ -1499,13 +1558,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D03E8B95-40CB-49F7-AF29-3A2B27B21A61}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="19.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1516,7 +1575,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1527,7 +1586,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1538,7 +1597,7 @@
         <v>1825</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1549,7 +1608,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1566,15 +1625,58 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C485CB82-74B9-4E1E-9CE3-715999920922}">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="C3">
+        <v>1825</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F19EA7F8-0885-4456-A6E5-96AB05BF51FA}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="25.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="40.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1585,7 +1687,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1596,7 +1698,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1607,7 +1709,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1624,16 +1726,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B47C19A-7081-4532-8CD1-2D1BC531686A}">
   <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="27.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1644,7 +1746,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1655,7 +1757,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1666,7 +1768,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1677,7 +1779,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1688,7 +1790,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -1699,7 +1801,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -1710,7 +1812,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -1721,7 +1823,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -1732,7 +1834,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -1743,7 +1845,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -1754,7 +1856,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>3</v>
       </c>
@@ -1763,108 +1865,6 @@
       </c>
       <c r="C12" t="s">
         <v>9</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4BADE6FB-E965-4263-BE22-5F02F8843366}">
-  <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="2" max="2" width="27" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="40.33203125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" t="s">
-        <v>69</v>
-      </c>
-      <c r="C4">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>20</v>
-      </c>
-      <c r="B5" t="s">
-        <v>21</v>
-      </c>
-      <c r="C5">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>20</v>
-      </c>
-      <c r="B6" t="s">
-        <v>22</v>
-      </c>
-      <c r="C6">
-        <v>10000</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>20</v>
-      </c>
-      <c r="B7" t="s">
-        <v>23</v>
-      </c>
-      <c r="C7">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>20</v>
-      </c>
-      <c r="B8" t="s">
-        <v>24</v>
-      </c>
-      <c r="C8">
-        <v>10000</v>
       </c>
     </row>
   </sheetData>
@@ -1873,15 +1873,15 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{531E32A4-7E13-4409-95B5-698B0506DEBB}">
-  <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4BADE6FB-E965-4263-BE22-5F02F8843366}">
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="26.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1892,70 +1892,81 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="C2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="C3" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C4" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+        <v>69</v>
+      </c>
+      <c r="C4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="B5" t="s">
-        <v>33</v>
-      </c>
-      <c r="C5" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+        <v>21</v>
+      </c>
+      <c r="C5">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="B6" t="s">
-        <v>35</v>
-      </c>
-      <c r="C6" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+        <v>22</v>
+      </c>
+      <c r="C6">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="B7" t="s">
-        <v>36</v>
-      </c>
-      <c r="C7" t="s">
-        <v>34</v>
+        <v>23</v>
+      </c>
+      <c r="C7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8">
+        <v>10000</v>
       </c>
     </row>
   </sheetData>
@@ -1964,13 +1975,17 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5034D7D-3DCC-4A67-A25F-FCA9FE48CDBA}">
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{531E32A4-7E13-4409-95B5-698B0506DEBB}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="26.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.08984375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>88</v>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>2</v>
@@ -1979,26 +1994,70 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>89</v>
+        <v>25</v>
       </c>
       <c r="C2" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>90</v>
-      </c>
-      <c r="C3">
-        <v>0</v>
+        <v>27</v>
+      </c>
+      <c r="C3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -2007,17 +2066,13 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70638D0A-5B68-4E82-8E59-C902079F733A}">
-  <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="2" max="2" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="70.77734375" bestFit="1" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5034D7D-3DCC-4A67-A25F-FCA9FE48CDBA}">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>88</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>2</v>
@@ -2026,125 +2081,26 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>38</v>
+        <v>89</v>
       </c>
       <c r="C2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="C3" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="C4" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="C5" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="C6" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="C7" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="C8" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="C9" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>98</v>
-      </c>
-      <c r="C10" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>99</v>
-      </c>
-      <c r="C11" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>3</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="C12" t="s">
-        <v>41</v>
+      <c r="B3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -2153,56 +2109,144 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B88D2545-36F8-47CF-B9C1-1EF7F48C6F22}">
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70638D0A-5B68-4E82-8E59-C902079F733A}">
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="20.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="33.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="70.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>101</v>
+        <v>38</v>
       </c>
       <c r="C2" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
-      <c r="B3" t="s">
-        <v>102</v>
+      <c r="B3" s="5" t="s">
+        <v>91</v>
       </c>
       <c r="C3" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" t="s">
-        <v>103</v>
+      <c r="B4" s="5" t="s">
+        <v>92</v>
       </c>
       <c r="C4" t="s">
-        <v>43</v>
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="C5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C6" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="C7" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="C8" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="C9" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="C10" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C11" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="C12" t="s">
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated Test Cases as per Report Analysis
</commit_message>
<xml_diff>
--- a/src/main/resources/Program_Field_Values_QA_org.xlsx
+++ b/src/main/resources/Program_Field_Values_QA_org.xlsx
@@ -1,29 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25831"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25928"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F91ACA1-67DA-4554-BB73-FC4EAC94C9E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDB06CBB-8325-488D-A530-68401074BDDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ProgramCreation_v" sheetId="22" r:id="rId1"/>
     <sheet name="ProgramEdition_v" sheetId="23" r:id="rId2"/>
     <sheet name="ProgramEditon_forCkEditor" sheetId="37" r:id="rId3"/>
     <sheet name="NewOrgAnnCreation_v" sheetId="24" r:id="rId4"/>
-    <sheet name="NewOrg2ndModal_v" sheetId="25" r:id="rId5"/>
-    <sheet name="NewOrgAnnEdition_v" sheetId="26" r:id="rId6"/>
-    <sheet name="NewOrgAppEddition_v" sheetId="27" r:id="rId7"/>
-    <sheet name="StandardAssurancesForm_v" sheetId="28" r:id="rId8"/>
-    <sheet name="ProgramApplicationForm_v" sheetId="29" r:id="rId9"/>
-    <sheet name="PaymentRequestSchedule_v" sheetId="30" r:id="rId10"/>
-    <sheet name="GrantCreation_v" sheetId="31" r:id="rId11"/>
-    <sheet name="Grant_Edition_v" sheetId="32" r:id="rId12"/>
-    <sheet name="StandAloneEdition_v" sheetId="33" r:id="rId13"/>
-    <sheet name="SiteVisitCreation_v" sheetId="34" r:id="rId14"/>
-    <sheet name="SiteVisitEdition_v" sheetId="35" r:id="rId15"/>
-    <sheet name="GeneralReviewForm_v" sheetId="36" r:id="rId16"/>
+    <sheet name="QA_OrgAnnCreation" sheetId="38" r:id="rId5"/>
+    <sheet name="NewOrg2ndModal_v" sheetId="25" r:id="rId6"/>
+    <sheet name="NewOrgAnnEdition_v" sheetId="26" r:id="rId7"/>
+    <sheet name="NewOrgAppEddition_v" sheetId="27" r:id="rId8"/>
+    <sheet name="StandardAssurancesForm_v" sheetId="28" r:id="rId9"/>
+    <sheet name="ProgramApplicationForm_v" sheetId="29" r:id="rId10"/>
+    <sheet name="PaymentRequestSchedule_v" sheetId="30" r:id="rId11"/>
+    <sheet name="GrantCreation_v" sheetId="31" r:id="rId12"/>
+    <sheet name="Grant_Edition_v" sheetId="32" r:id="rId13"/>
+    <sheet name="StandAloneEdition_v" sheetId="33" r:id="rId14"/>
+    <sheet name="SiteVisitCreation_v" sheetId="34" r:id="rId15"/>
+    <sheet name="SiteVisitEdition_v" sheetId="35" r:id="rId16"/>
+    <sheet name="GeneralReviewForm_v" sheetId="36" r:id="rId17"/>
   </sheets>
   <calcPr calcId="179017"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="132">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -875,6 +876,152 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70638D0A-5B68-4E82-8E59-C902079F733A}">
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="14.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="70.81640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="C3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="C4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="C5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C6" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="C7" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="C8" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="C9" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="C10" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C11" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="C12" t="s">
+        <v>41</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B88D2545-36F8-47CF-B9C1-1EF7F48C6F22}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -932,7 +1079,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8CB8E10-5A8B-4AF3-AF66-F1E9AA7C9BBC}">
   <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1045,7 +1192,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55BEB37B-B28E-4F60-BECB-CD35E74B4C36}">
   <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1191,7 +1338,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82865F4C-F847-4F90-8B11-C831BFCC23C2}">
   <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1271,7 +1418,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDDAC24B-DC90-49E6-BD31-6F210026CA6D}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1329,7 +1476,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6F7845C-214C-4C02-A5F4-6F38FB46E35D}">
   <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1431,7 +1578,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE64D93B-66B6-48F6-99BC-E4BA23590E06}">
   <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1727,6 +1874,54 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C0E25E5-8973-4E31-A3CE-0B2930FA70C8}">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="7.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40.90625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="C2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="C3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B47C19A-7081-4532-8CD1-2D1BC531686A}">
   <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1872,7 +2067,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4BADE6FB-E965-4263-BE22-5F02F8843366}">
   <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1974,7 +2169,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{531E32A4-7E13-4409-95B5-698B0506DEBB}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -2065,7 +2260,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5034D7D-3DCC-4A67-A25F-FCA9FE48CDBA}">
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -2106,150 +2301,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70638D0A-5B68-4E82-8E59-C902079F733A}">
-  <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="2" max="2" width="14.90625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="70.81640625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="C3" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="C4" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="C5" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="C6" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="C7" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="C8" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="C9" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>98</v>
-      </c>
-      <c r="C10" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>99</v>
-      </c>
-      <c r="C11" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
-        <v>3</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="C12" t="s">
-        <v>41</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Update Test cases as per analysis and Newly added TC in SendEmail LWC
</commit_message>
<xml_diff>
--- a/src/main/resources/Program_Field_Values_QA_org.xlsx
+++ b/src/main/resources/Program_Field_Values_QA_org.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26026"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDB06CBB-8325-488D-A530-68401074BDDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38CA6A46-6FD4-4284-948B-C917407CB8D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="10" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ProgramCreation_v" sheetId="22" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="132">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -80,9 +80,6 @@
     <t>IsProgramIncomeAnticipated__c</t>
   </si>
   <si>
-    <t>WBSRequired__c</t>
-  </si>
-  <si>
     <t>AreExpensesBuildIUpLevel__c</t>
   </si>
   <si>
@@ -432,6 +429,9 @@
   </si>
   <si>
     <t>Test Automation Organization</t>
+  </si>
+  <si>
+    <t>CalReportingEndDate__c</t>
   </si>
 </sst>
 </file>
@@ -808,10 +808,10 @@
         <v>3</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C2" t="s">
         <v>71</v>
-      </c>
-      <c r="C2" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
@@ -819,7 +819,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C3" t="s">
         <v>4</v>
@@ -830,10 +830,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
@@ -841,7 +841,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C5" t="s">
         <v>9</v>
@@ -852,7 +852,7 @@
         <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C6" t="s">
         <v>9</v>
@@ -863,7 +863,7 @@
         <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C7" t="s">
         <v>9</v>
@@ -900,10 +900,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C2" t="s">
         <v>38</v>
-      </c>
-      <c r="C2" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
@@ -911,10 +911,10 @@
         <v>3</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
@@ -922,10 +922,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
@@ -933,10 +933,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
@@ -944,10 +944,10 @@
         <v>3</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
@@ -955,10 +955,10 @@
         <v>3</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
@@ -966,10 +966,10 @@
         <v>3</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
@@ -977,10 +977,10 @@
         <v>3</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
@@ -988,10 +988,10 @@
         <v>3</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
@@ -999,10 +999,10 @@
         <v>3</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
@@ -1010,10 +1010,10 @@
         <v>3</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C12" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -1023,10 +1023,10 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B88D2545-36F8-47CF-B9C1-1EF7F48C6F22}">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="20.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.453125" customWidth="1"/>
     <col min="3" max="3" width="33.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1046,10 +1046,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
@@ -1057,10 +1057,10 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
@@ -1068,14 +1068,26 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C4" t="s">
-        <v>43</v>
+        <v>42</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>131</v>
+      </c>
+      <c r="C5">
+        <v>300</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1104,10 +1116,10 @@
         <v>3</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
@@ -1115,10 +1127,10 @@
         <v>3</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
@@ -1126,7 +1138,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -1137,7 +1149,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C5">
         <v>365</v>
@@ -1148,10 +1160,10 @@
         <v>3</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
@@ -1159,10 +1171,10 @@
         <v>3</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C7" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
@@ -1170,10 +1182,10 @@
         <v>3</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
@@ -1181,10 +1193,10 @@
         <v>3</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C9" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
   </sheetData>
@@ -1194,7 +1206,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55BEB37B-B28E-4F60-BECB-CD35E74B4C36}">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="27.90625" bestFit="1" customWidth="1"/>
@@ -1250,7 +1262,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C5" t="s">
         <v>9</v>
@@ -1261,7 +1273,7 @@
         <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C6" t="s">
         <v>9</v>
@@ -1294,7 +1306,7 @@
         <v>3</v>
       </c>
       <c r="B9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C9" t="s">
         <v>9</v>
@@ -1305,7 +1317,7 @@
         <v>3</v>
       </c>
       <c r="B10" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C10" t="s">
         <v>9</v>
@@ -1316,20 +1328,9 @@
         <v>3</v>
       </c>
       <c r="B11" t="s">
-        <v>14</v>
+        <v>65</v>
       </c>
       <c r="C11" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
-        <v>3</v>
-      </c>
-      <c r="B12" t="s">
-        <v>66</v>
-      </c>
-      <c r="C12" t="s">
         <v>9</v>
       </c>
     </row>
@@ -1363,10 +1364,10 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
@@ -1374,10 +1375,10 @@
         <v>5</v>
       </c>
       <c r="B3" t="s">
+        <v>110</v>
+      </c>
+      <c r="C3" t="s">
         <v>111</v>
-      </c>
-      <c r="C3" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
@@ -1385,10 +1386,10 @@
         <v>5</v>
       </c>
       <c r="B4" t="s">
+        <v>112</v>
+      </c>
+      <c r="C4" t="s">
         <v>113</v>
-      </c>
-      <c r="C4" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
@@ -1396,7 +1397,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C5">
         <v>1234</v>
@@ -1404,13 +1405,13 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C6">
-        <v>3650</v>
+        <v>330</v>
       </c>
     </row>
   </sheetData>
@@ -1443,10 +1444,10 @@
         <v>3</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
@@ -1454,10 +1455,10 @@
         <v>3</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
@@ -1465,10 +1466,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -1501,7 +1502,7 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C2">
         <v>365</v>
@@ -1512,7 +1513,7 @@
         <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C3">
         <v>455</v>
@@ -1523,10 +1524,10 @@
         <v>5</v>
       </c>
       <c r="B4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C4" t="s">
         <v>54</v>
-      </c>
-      <c r="C4" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
@@ -1534,10 +1535,10 @@
         <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
@@ -1545,10 +1546,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
+        <v>56</v>
+      </c>
+      <c r="C6" t="s">
         <v>57</v>
-      </c>
-      <c r="C6" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
@@ -1556,10 +1557,10 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
+        <v>58</v>
+      </c>
+      <c r="C7" t="s">
         <v>59</v>
-      </c>
-      <c r="C7" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
@@ -1567,10 +1568,10 @@
         <v>5</v>
       </c>
       <c r="B8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C8" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
   </sheetData>
@@ -1603,10 +1604,10 @@
         <v>3</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
@@ -1614,10 +1615,10 @@
         <v>3</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
@@ -1625,10 +1626,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
@@ -1636,10 +1637,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
@@ -1647,10 +1648,10 @@
         <v>3</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
@@ -1658,10 +1659,10 @@
         <v>3</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
@@ -1669,10 +1670,10 @@
         <v>3</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
@@ -1680,10 +1681,10 @@
         <v>3</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
@@ -1691,10 +1692,10 @@
         <v>3</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
   </sheetData>
@@ -1727,7 +1728,7 @@
         <v>3</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -1738,7 +1739,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C3">
         <v>1825</v>
@@ -1749,10 +1750,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C4" t="s">
         <v>74</v>
-      </c>
-      <c r="C4" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
@@ -1760,10 +1761,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>
@@ -1792,7 +1793,7 @@
         <v>3</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -1803,7 +1804,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C3">
         <v>1825</v>
@@ -1839,10 +1840,10 @@
         <v>3</v>
       </c>
       <c r="B2" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="C2" t="s">
         <v>77</v>
-      </c>
-      <c r="C2" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
@@ -1850,10 +1851,10 @@
         <v>3</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
@@ -1861,7 +1862,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C4" t="s">
         <v>10</v>
@@ -1899,10 +1900,10 @@
         <v>3</v>
       </c>
       <c r="B2" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="C2" t="s">
         <v>77</v>
-      </c>
-      <c r="C2" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
@@ -1910,7 +1911,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C3" t="s">
         <v>10</v>
@@ -1946,7 +1947,7 @@
         <v>3</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C2" t="s">
         <v>9</v>
@@ -1957,7 +1958,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C3" t="s">
         <v>9</v>
@@ -1968,7 +1969,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C4" t="s">
         <v>9</v>
@@ -1979,7 +1980,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C5" t="s">
         <v>9</v>
@@ -1990,7 +1991,7 @@
         <v>3</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C6" t="s">
         <v>9</v>
@@ -2001,7 +2002,7 @@
         <v>3</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C7" t="s">
         <v>9</v>
@@ -2012,7 +2013,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C8" t="s">
         <v>9</v>
@@ -2023,7 +2024,7 @@
         <v>3</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C9" t="s">
         <v>9</v>
@@ -2034,7 +2035,7 @@
         <v>3</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C10" t="s">
         <v>9</v>
@@ -2045,7 +2046,7 @@
         <v>3</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C11" t="s">
         <v>9</v>
@@ -2056,7 +2057,7 @@
         <v>3</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C12" t="s">
         <v>9</v>
@@ -2092,7 +2093,7 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C2" t="s">
         <v>6</v>
@@ -2103,10 +2104,10 @@
         <v>5</v>
       </c>
       <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
         <v>18</v>
-      </c>
-      <c r="C3" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
@@ -2114,7 +2115,7 @@
         <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C4">
         <v>20</v>
@@ -2122,10 +2123,10 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" t="s">
         <v>20</v>
-      </c>
-      <c r="B5" t="s">
-        <v>21</v>
       </c>
       <c r="C5">
         <v>1000</v>
@@ -2133,10 +2134,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C6">
         <v>10000</v>
@@ -2144,10 +2145,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C7">
         <v>2</v>
@@ -2155,10 +2156,10 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B8" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C8">
         <v>10000</v>
@@ -2194,10 +2195,10 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" t="s">
         <v>25</v>
-      </c>
-      <c r="C2" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
@@ -2205,54 +2206,54 @@
         <v>5</v>
       </c>
       <c r="B3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" t="s">
         <v>27</v>
-      </c>
-      <c r="C3" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" t="s">
         <v>29</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>30</v>
-      </c>
-      <c r="C4" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B5" t="s">
         <v>32</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>33</v>
-      </c>
-      <c r="C5" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C7" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -2267,7 +2268,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>2</v>
@@ -2281,10 +2282,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
@@ -2292,7 +2293,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C3">
         <v>0</v>

</xml_diff>

<commit_message>
update test case in sanity QA and Test5 org
</commit_message>
<xml_diff>
--- a/src/main/resources/Program_Field_Values_QA_org.xlsx
+++ b/src/main/resources/Program_Field_Values_QA_org.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26130"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38CA6A46-6FD4-4284-948B-C917407CB8D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55E89162-39B8-4E39-8E43-AE820E1B8FB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="10" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="10" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ProgramCreation_v" sheetId="22" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="133">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -432,6 +432,9 @@
   </si>
   <si>
     <t>CalReportingEndDate__c</t>
+  </si>
+  <si>
+    <t>PG-A11-0038</t>
   </si>
 </sst>
 </file>
@@ -1185,7 +1188,7 @@
         <v>69</v>
       </c>
       <c r="C8" t="s">
-        <v>71</v>
+        <v>132</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
updated test cases in dynamic form as per report analysis
</commit_message>
<xml_diff>
--- a/src/main/resources/Program_Field_Values_QA_org.xlsx
+++ b/src/main/resources/Program_Field_Values_QA_org.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26227"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55E89162-39B8-4E39-8E43-AE820E1B8FB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D9D497C-ECDC-4805-A55D-7600F9D74194}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="10" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ProgramCreation_v" sheetId="22" r:id="rId1"/>

</xml_diff>

<commit_message>
Changes in e-grid table module
</commit_message>
<xml_diff>
--- a/src/main/resources/Program_Field_Values_QA_org.xlsx
+++ b/src/main/resources/Program_Field_Values_QA_org.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26529"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCC8DBB5-B43C-40EF-B70C-6A379F3B9FE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8F399F1-1705-4EAB-8EC9-9630F190E9EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="9" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ProgramCreation_v" sheetId="22" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="134">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -435,6 +435,9 @@
   </si>
   <si>
     <t>Automation Direct Grant</t>
+  </si>
+  <si>
+    <t>Automation Program For Test</t>
   </si>
 </sst>
 </file>
@@ -789,13 +792,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E83D430-2DDF-4C96-A733-8F6A18593E6C}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -806,7 +809,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -814,10 +817,10 @@
         <v>69</v>
       </c>
       <c r="C2" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -828,7 +831,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -839,7 +842,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -850,7 +853,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -861,7 +864,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -881,13 +884,13 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70638D0A-5B68-4E82-8E59-C902079F733A}">
   <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="14.90625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="70.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="70.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -898,7 +901,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -909,7 +912,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -920,7 +923,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -931,7 +934,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -942,7 +945,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -953,7 +956,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -964,7 +967,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -975,7 +978,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -986,7 +989,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -997,7 +1000,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -1008,7 +1011,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>3</v>
       </c>
@@ -1027,13 +1030,13 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B88D2545-36F8-47CF-B9C1-1EF7F48C6F22}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="23.453125" customWidth="1"/>
-    <col min="3" max="3" width="33.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.44140625" customWidth="1"/>
+    <col min="3" max="3" width="33.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1044,7 +1047,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1055,7 +1058,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1066,7 +1069,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1077,7 +1080,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1097,13 +1100,13 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8CB8E10-5A8B-4AF3-AF66-F1E9AA7C9BBC}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="27.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="39.81640625" customWidth="1"/>
+    <col min="2" max="2" width="27.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="39.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1114,7 +1117,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1125,7 +1128,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1136,7 +1139,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1147,7 +1150,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1158,7 +1161,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -1169,7 +1172,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -1180,7 +1183,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -1191,7 +1194,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -1210,13 +1213,13 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55BEB37B-B28E-4F60-BECB-CD35E74B4C36}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="27.90625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1227,7 +1230,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1238,7 +1241,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1249,7 +1252,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1260,7 +1263,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1271,7 +1274,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -1282,7 +1285,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -1293,7 +1296,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -1304,7 +1307,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -1315,7 +1318,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -1326,7 +1329,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -1345,13 +1348,13 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82865F4C-F847-4F90-8B11-C831BFCC23C2}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="30" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1362,7 +1365,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1373,7 +1376,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -1384,7 +1387,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -1395,7 +1398,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -1406,7 +1409,7 @@
         <v>1234</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>28</v>
       </c>
@@ -1425,13 +1428,13 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDDAC24B-DC90-49E6-BD31-6F210026CA6D}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="20.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="25.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1442,7 +1445,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1453,7 +1456,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1464,7 +1467,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1483,13 +1486,13 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6F7845C-214C-4C02-A5F4-6F38FB46E35D}">
   <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="33.90625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="41.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="33.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1500,7 +1503,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1511,7 +1514,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -1522,7 +1525,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -1533,7 +1536,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -1544,7 +1547,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -1555,7 +1558,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -1566,7 +1569,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>5</v>
       </c>
@@ -1585,13 +1588,13 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE64D93B-66B6-48F6-99BC-E4BA23590E06}">
   <dimension ref="A1:C10"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="23" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1602,7 +1605,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -1613,7 +1616,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -1624,7 +1627,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -1635,7 +1638,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -1646,7 +1649,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
@@ -1657,7 +1660,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>3</v>
       </c>
@@ -1668,7 +1671,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>3</v>
       </c>
@@ -1679,7 +1682,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>3</v>
       </c>
@@ -1690,7 +1693,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>3</v>
       </c>
@@ -1709,13 +1712,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D03E8B95-40CB-49F7-AF29-3A2B27B21A61}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="19.6328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1726,7 +1729,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1737,7 +1740,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1748,7 +1751,7 @@
         <v>1825</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1759,7 +1762,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1778,9 +1781,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C485CB82-74B9-4E1E-9CE3-715999920922}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1791,7 +1794,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1802,7 +1805,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1821,13 +1824,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F19EA7F8-0885-4456-A6E5-96AB05BF51FA}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="25.36328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="40.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1838,7 +1841,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1849,7 +1852,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1860,7 +1863,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1880,14 +1883,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C0E25E5-8973-4E31-A3CE-0B2930FA70C8}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="40.90625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1898,7 +1901,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1909,7 +1912,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1928,13 +1931,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B47C19A-7081-4532-8CD1-2D1BC531686A}">
   <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="27.6328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1945,7 +1948,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1956,7 +1959,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1967,7 +1970,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1978,7 +1981,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1989,7 +1992,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -2000,7 +2003,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -2011,7 +2014,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -2022,7 +2025,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -2033,7 +2036,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -2044,7 +2047,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -2055,7 +2058,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>3</v>
       </c>
@@ -2074,13 +2077,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4BADE6FB-E965-4263-BE22-5F02F8843366}">
   <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="27" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="40.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2091,7 +2094,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -2102,7 +2105,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -2113,7 +2116,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -2124,7 +2127,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>19</v>
       </c>
@@ -2135,7 +2138,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>19</v>
       </c>
@@ -2146,7 +2149,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -2157,7 +2160,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -2176,13 +2179,13 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{531E32A4-7E13-4409-95B5-698B0506DEBB}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="26.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2193,7 +2196,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -2204,7 +2207,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -2215,7 +2218,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>28</v>
       </c>
@@ -2226,7 +2229,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>31</v>
       </c>
@@ -2237,7 +2240,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>31</v>
       </c>
@@ -2248,7 +2251,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>31</v>
       </c>
@@ -2267,9 +2270,9 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5034D7D-3DCC-4A67-A25F-FCA9FE48CDBA}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>86</v>
       </c>
@@ -2280,7 +2283,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2291,7 +2294,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>

</xml_diff>

<commit_message>
create record for pdfxlsscenario
</commit_message>
<xml_diff>
--- a/src/main/resources/Program_Field_Values_QA_org.xlsx
+++ b/src/main/resources/Program_Field_Values_QA_org.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26529"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCC8DBB5-B43C-40EF-B70C-6A379F3B9FE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BCDAF92-AF21-4D65-93D2-9750AE6CAC75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="9" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ProgramCreation_v" sheetId="22" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="134">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -435,6 +435,9 @@
   </si>
   <si>
     <t>Automation Direct Grant</t>
+  </si>
+  <si>
+    <t>Automation Program For Test</t>
   </si>
 </sst>
 </file>
@@ -814,7 +817,7 @@
         <v>69</v>
       </c>
       <c r="C2" t="s">
-        <v>70</v>
+        <v>133</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Updated Expression Builder module
</commit_message>
<xml_diff>
--- a/src/main/resources/Program_Field_Values_QA_org.xlsx
+++ b/src/main/resources/Program_Field_Values_QA_org.xlsx
@@ -1,30 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26529"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26626"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8F399F1-1705-4EAB-8EC9-9630F190E9EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3AB2BD1-FD21-481F-9093-1E642F7175B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="ProgramCreation_v" sheetId="22" r:id="rId1"/>
-    <sheet name="ProgramEdition_v" sheetId="23" r:id="rId2"/>
-    <sheet name="ProgramEditon_forCkEditor" sheetId="37" r:id="rId3"/>
-    <sheet name="NewOrgAnnCreation_v" sheetId="24" r:id="rId4"/>
-    <sheet name="QA_OrgAnnCreation" sheetId="38" r:id="rId5"/>
-    <sheet name="NewOrg2ndModal_v" sheetId="25" r:id="rId6"/>
-    <sheet name="NewOrgAnnEdition_v" sheetId="26" r:id="rId7"/>
-    <sheet name="NewOrgAppEddition_v" sheetId="27" r:id="rId8"/>
-    <sheet name="StandardAssurancesForm_v" sheetId="28" r:id="rId9"/>
-    <sheet name="ProgramApplicationForm_v" sheetId="29" r:id="rId10"/>
-    <sheet name="PaymentRequestSchedule_v" sheetId="30" r:id="rId11"/>
-    <sheet name="GrantCreation_v" sheetId="31" r:id="rId12"/>
-    <sheet name="Grant_Edition_v" sheetId="32" r:id="rId13"/>
-    <sheet name="StandAloneEdition_v" sheetId="33" r:id="rId14"/>
-    <sheet name="SiteVisitCreation_v" sheetId="34" r:id="rId15"/>
-    <sheet name="SiteVisitEdition_v" sheetId="35" r:id="rId16"/>
-    <sheet name="GeneralReviewForm_v" sheetId="36" r:id="rId17"/>
+    <sheet name="StaticRecordProgramCreation" sheetId="39" r:id="rId1"/>
+    <sheet name="ProgramCreation_v" sheetId="22" r:id="rId2"/>
+    <sheet name="ProgramEdition_v" sheetId="23" r:id="rId3"/>
+    <sheet name="ProgramEditon_forCkEditor" sheetId="37" r:id="rId4"/>
+    <sheet name="NewOrgAnnCreation_v" sheetId="24" r:id="rId5"/>
+    <sheet name="QA_OrgAnnCreation" sheetId="38" r:id="rId6"/>
+    <sheet name="NewOrg2ndModal_v" sheetId="25" r:id="rId7"/>
+    <sheet name="NewOrgAnnEdition_v" sheetId="26" r:id="rId8"/>
+    <sheet name="NewOrgAppEddition_v" sheetId="27" r:id="rId9"/>
+    <sheet name="StandardAssurancesForm_v" sheetId="28" r:id="rId10"/>
+    <sheet name="ProgramApplicationForm_v" sheetId="29" r:id="rId11"/>
+    <sheet name="PaymentRequestSchedule_v" sheetId="30" r:id="rId12"/>
+    <sheet name="GrantCreation_v" sheetId="31" r:id="rId13"/>
+    <sheet name="Grant_Edition_v" sheetId="32" r:id="rId14"/>
+    <sheet name="StandAloneEdition_v" sheetId="33" r:id="rId15"/>
+    <sheet name="SiteVisitCreation_v" sheetId="34" r:id="rId16"/>
+    <sheet name="SiteVisitEdition_v" sheetId="35" r:id="rId17"/>
+    <sheet name="GeneralReviewForm_v" sheetId="36" r:id="rId18"/>
   </sheets>
   <calcPr calcId="179017"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="134">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -790,6 +791,969 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9504DEE-61CE-471E-847C-6DA763CE3AF2}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="30.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="45.21875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>63</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>64</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>65</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>66</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5034D7D-3DCC-4A67-A25F-FCA9FE48CDBA}">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>86</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>88</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70638D0A-5B68-4E82-8E59-C902079F733A}">
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="70.77734375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="C3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="C4" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="C5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="C6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="C7" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C8" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="C9" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="C10" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="C11" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="C12" t="s">
+        <v>40</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B88D2545-36F8-47CF-B9C1-1EF7F48C6F22}">
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="23.44140625" customWidth="1"/>
+    <col min="3" max="3" width="33.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>101</v>
+      </c>
+      <c r="C4" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>130</v>
+      </c>
+      <c r="C5">
+        <v>300</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8CB8E10-5A8B-4AF3-AF66-F1E9AA7C9BBC}">
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="27.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="39.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C5">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="C6" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="C7" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="C8" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="C9" t="s">
+        <v>129</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55BEB37B-B28E-4F60-BECB-CD35E74B4C36}">
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="27.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.77734375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>48</v>
+      </c>
+      <c r="C6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
+        <v>49</v>
+      </c>
+      <c r="C10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82865F4C-F847-4F90-8B11-C831BFCC23C2}">
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="30" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.5546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" t="s">
+        <v>109</v>
+      </c>
+      <c r="C3" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" t="s">
+        <v>111</v>
+      </c>
+      <c r="C4" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" t="s">
+        <v>113</v>
+      </c>
+      <c r="C5">
+        <v>1234</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" t="s">
+        <v>114</v>
+      </c>
+      <c r="C6">
+        <v>330</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDDAC24B-DC90-49E6-BD31-6F210026CA6D}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="C2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="C3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="C4" t="s">
+        <v>51</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6F7845C-214C-4C02-A5F4-6F38FB46E35D}">
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="33.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41.21875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>118</v>
+      </c>
+      <c r="C2">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" t="s">
+        <v>119</v>
+      </c>
+      <c r="C3">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C4" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" t="s">
+        <v>54</v>
+      </c>
+      <c r="C5" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>55</v>
+      </c>
+      <c r="C6" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" t="s">
+        <v>57</v>
+      </c>
+      <c r="C7" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" t="s">
+        <v>59</v>
+      </c>
+      <c r="C8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE64D93B-66B6-48F6-99BC-E4BA23590E06}">
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="23" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.21875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>110</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E83D430-2DDF-4C96-A733-8F6A18593E6C}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -881,835 +1845,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70638D0A-5B68-4E82-8E59-C902079F733A}">
-  <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="2" max="2" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="70.77734375" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C2" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="C3" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="C4" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="C5" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="C6" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="C7" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="C8" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="C9" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="C10" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="C11" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>3</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>98</v>
-      </c>
-      <c r="C12" t="s">
-        <v>40</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B88D2545-36F8-47CF-B9C1-1EF7F48C6F22}">
-  <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="2" max="2" width="23.44140625" customWidth="1"/>
-    <col min="3" max="3" width="33.44140625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>99</v>
-      </c>
-      <c r="C2" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>100</v>
-      </c>
-      <c r="C3" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>101</v>
-      </c>
-      <c r="C4" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" t="s">
-        <v>130</v>
-      </c>
-      <c r="C5">
-        <v>300</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8CB8E10-5A8B-4AF3-AF66-F1E9AA7C9BBC}">
-  <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="2" max="2" width="27.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="39.77734375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="C3" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="C4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>104</v>
-      </c>
-      <c r="C5">
-        <v>365</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>105</v>
-      </c>
-      <c r="C6" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="C7" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="C8" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>107</v>
-      </c>
-      <c r="C9" t="s">
-        <v>129</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55BEB37B-B28E-4F60-BECB-CD35E74B4C36}">
-  <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="2" max="2" width="27.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.77734375" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" t="s">
-        <v>48</v>
-      </c>
-      <c r="C6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" t="s">
-        <v>8</v>
-      </c>
-      <c r="C7" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" t="s">
-        <v>7</v>
-      </c>
-      <c r="C8" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" t="s">
-        <v>14</v>
-      </c>
-      <c r="C9" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" t="s">
-        <v>49</v>
-      </c>
-      <c r="C10" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" t="s">
-        <v>64</v>
-      </c>
-      <c r="C11" t="s">
-        <v>9</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82865F4C-F847-4F90-8B11-C831BFCC23C2}">
-  <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="2" max="2" width="30" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.5546875" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>108</v>
-      </c>
-      <c r="C2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" t="s">
-        <v>109</v>
-      </c>
-      <c r="C3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" t="s">
-        <v>111</v>
-      </c>
-      <c r="C4" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" t="s">
-        <v>113</v>
-      </c>
-      <c r="C5">
-        <v>1234</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>28</v>
-      </c>
-      <c r="B6" t="s">
-        <v>114</v>
-      </c>
-      <c r="C6">
-        <v>330</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDDAC24B-DC90-49E6-BD31-6F210026CA6D}">
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="25.6640625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>115</v>
-      </c>
-      <c r="C2" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="C3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="C4" t="s">
-        <v>51</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6F7845C-214C-4C02-A5F4-6F38FB46E35D}">
-  <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="2" max="2" width="33.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="41.21875" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>118</v>
-      </c>
-      <c r="C2">
-        <v>365</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" t="s">
-        <v>119</v>
-      </c>
-      <c r="C3">
-        <v>455</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" t="s">
-        <v>52</v>
-      </c>
-      <c r="C4" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" t="s">
-        <v>54</v>
-      </c>
-      <c r="C5" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>5</v>
-      </c>
-      <c r="B6" t="s">
-        <v>55</v>
-      </c>
-      <c r="C6" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>5</v>
-      </c>
-      <c r="B7" t="s">
-        <v>57</v>
-      </c>
-      <c r="C7" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B8" t="s">
-        <v>59</v>
-      </c>
-      <c r="C8" t="s">
-        <v>53</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE64D93B-66B6-48F6-99BC-E4BA23590E06}">
-  <dimension ref="A1:C10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="2" max="2" width="23" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.21875" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>110</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D03E8B95-40CB-49F7-AF29-3A2B27B21A61}">
   <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1778,7 +1914,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C485CB82-74B9-4E1E-9CE3-715999920922}">
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1821,7 +1957,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F19EA7F8-0885-4456-A6E5-96AB05BF51FA}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1880,7 +2016,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C0E25E5-8973-4E31-A3CE-0B2930FA70C8}">
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1928,7 +2064,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B47C19A-7081-4532-8CD1-2D1BC531686A}">
   <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2074,7 +2210,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4BADE6FB-E965-4263-BE22-5F02F8843366}">
   <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2176,7 +2312,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{531E32A4-7E13-4409-95B5-698B0506DEBB}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2265,47 +2401,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5034D7D-3DCC-4A67-A25F-FCA9FE48CDBA}">
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>86</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>87</v>
-      </c>
-      <c r="C2" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>88</v>
-      </c>
-      <c r="C3">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
changes in Sanity TC
</commit_message>
<xml_diff>
--- a/src/main/resources/Program_Field_Values_QA_org.xlsx
+++ b/src/main/resources/Program_Field_Values_QA_org.xlsx
@@ -1,31 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26626"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26731"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3AB2BD1-FD21-481F-9093-1E642F7175B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A0EA79C-71C3-4653-BE67-B0EF940C36CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="StaticRecordProgramCreation" sheetId="39" r:id="rId1"/>
-    <sheet name="ProgramCreation_v" sheetId="22" r:id="rId2"/>
-    <sheet name="ProgramEdition_v" sheetId="23" r:id="rId3"/>
-    <sheet name="ProgramEditon_forCkEditor" sheetId="37" r:id="rId4"/>
-    <sheet name="NewOrgAnnCreation_v" sheetId="24" r:id="rId5"/>
-    <sheet name="QA_OrgAnnCreation" sheetId="38" r:id="rId6"/>
-    <sheet name="NewOrg2ndModal_v" sheetId="25" r:id="rId7"/>
-    <sheet name="NewOrgAnnEdition_v" sheetId="26" r:id="rId8"/>
-    <sheet name="NewOrgAppEddition_v" sheetId="27" r:id="rId9"/>
-    <sheet name="StandardAssurancesForm_v" sheetId="28" r:id="rId10"/>
-    <sheet name="ProgramApplicationForm_v" sheetId="29" r:id="rId11"/>
-    <sheet name="PaymentRequestSchedule_v" sheetId="30" r:id="rId12"/>
-    <sheet name="GrantCreation_v" sheetId="31" r:id="rId13"/>
-    <sheet name="Grant_Edition_v" sheetId="32" r:id="rId14"/>
-    <sheet name="StandAloneEdition_v" sheetId="33" r:id="rId15"/>
-    <sheet name="SiteVisitCreation_v" sheetId="34" r:id="rId16"/>
-    <sheet name="SiteVisitEdition_v" sheetId="35" r:id="rId17"/>
-    <sheet name="GeneralReviewForm_v" sheetId="36" r:id="rId18"/>
+    <sheet name="ProgramCreation_v_for_Ann" sheetId="40" r:id="rId2"/>
+    <sheet name="ProgramCreation_v" sheetId="22" r:id="rId3"/>
+    <sheet name="ProgramEdition_v" sheetId="23" r:id="rId4"/>
+    <sheet name="ProgramEditon_forCkEditor" sheetId="37" r:id="rId5"/>
+    <sheet name="NewOrgAnnCreation_v" sheetId="24" r:id="rId6"/>
+    <sheet name="QA_OrgAnnCreation" sheetId="38" r:id="rId7"/>
+    <sheet name="NewOrg2ndModal_v" sheetId="25" r:id="rId8"/>
+    <sheet name="NewOrgAnnEdition_v" sheetId="26" r:id="rId9"/>
+    <sheet name="NewOrgAppEddition_v" sheetId="27" r:id="rId10"/>
+    <sheet name="StandardAssurancesForm_v" sheetId="28" r:id="rId11"/>
+    <sheet name="ProgramApplicationForm_v" sheetId="29" r:id="rId12"/>
+    <sheet name="PaymentRequestSchedule_v" sheetId="30" r:id="rId13"/>
+    <sheet name="GrantCreation_v" sheetId="31" r:id="rId14"/>
+    <sheet name="Grant_Edition_v" sheetId="32" r:id="rId15"/>
+    <sheet name="StandAloneEdition_v" sheetId="33" r:id="rId16"/>
+    <sheet name="SiteVisitCreation_v" sheetId="34" r:id="rId17"/>
+    <sheet name="SiteVisitEdition_v" sheetId="35" r:id="rId18"/>
+    <sheet name="GeneralReviewForm_v" sheetId="36" r:id="rId19"/>
   </sheets>
   <calcPr calcId="179017"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="135">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -439,6 +440,9 @@
   </si>
   <si>
     <t>Automation Program For Test</t>
+  </si>
+  <si>
+    <t>Automation Program For Announcement</t>
   </si>
 </sst>
 </file>
@@ -793,13 +797,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9504DEE-61CE-471E-847C-6DA763CE3AF2}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="30.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="45.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="45.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -810,7 +814,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -821,7 +825,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -832,7 +836,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -843,7 +847,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -854,7 +858,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -865,7 +869,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -883,13 +887,17 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5034D7D-3DCC-4A67-A25F-FCA9FE48CDBA}">
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{531E32A4-7E13-4409-95B5-698B0506DEBB}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="26.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.08984375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>86</v>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>2</v>
@@ -898,26 +906,70 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>87</v>
+        <v>24</v>
       </c>
       <c r="C2" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>88</v>
-      </c>
-      <c r="C3">
-        <v>0</v>
+        <v>26</v>
+      </c>
+      <c r="C3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" t="s">
+        <v>34</v>
+      </c>
+      <c r="C6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" t="s">
+        <v>35</v>
+      </c>
+      <c r="C7" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -926,17 +978,13 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70638D0A-5B68-4E82-8E59-C902079F733A}">
-  <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="2" max="2" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="70.77734375" bestFit="1" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5034D7D-3DCC-4A67-A25F-FCA9FE48CDBA}">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>86</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>2</v>
@@ -945,125 +993,26 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>37</v>
+        <v>87</v>
       </c>
       <c r="C2" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="C3" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="C4" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="C5" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="C6" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="C7" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="C8" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="C9" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="C10" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="C11" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>3</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>98</v>
-      </c>
-      <c r="C12" t="s">
-        <v>40</v>
+      <c r="B3" t="s">
+        <v>88</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1072,15 +1021,161 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70638D0A-5B68-4E82-8E59-C902079F733A}">
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="14.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="70.81640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="C3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="C4" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="C5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="C6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="C7" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C8" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="C9" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="C10" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="C11" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="C12" t="s">
+        <v>40</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B88D2545-36F8-47CF-B9C1-1EF7F48C6F22}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="23.44140625" customWidth="1"/>
-    <col min="3" max="3" width="33.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.453125" customWidth="1"/>
+    <col min="3" max="3" width="33.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1091,7 +1186,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1102,7 +1197,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1113,7 +1208,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1124,7 +1219,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1141,16 +1236,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8CB8E10-5A8B-4AF3-AF66-F1E9AA7C9BBC}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="27.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="39.77734375" customWidth="1"/>
+    <col min="2" max="2" width="27.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="39.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1161,7 +1256,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1172,7 +1267,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1183,7 +1278,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1194,7 +1289,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1205,7 +1300,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -1216,7 +1311,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -1227,7 +1322,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -1238,7 +1333,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -1247,141 +1342,6 @@
       </c>
       <c r="C9" t="s">
         <v>129</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55BEB37B-B28E-4F60-BECB-CD35E74B4C36}">
-  <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="2" max="2" width="27.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.77734375" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" t="s">
-        <v>48</v>
-      </c>
-      <c r="C6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" t="s">
-        <v>8</v>
-      </c>
-      <c r="C7" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" t="s">
-        <v>7</v>
-      </c>
-      <c r="C8" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" t="s">
-        <v>14</v>
-      </c>
-      <c r="C9" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" t="s">
-        <v>49</v>
-      </c>
-      <c r="C10" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" t="s">
-        <v>64</v>
-      </c>
-      <c r="C11" t="s">
-        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -1390,15 +1350,15 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82865F4C-F847-4F90-8B11-C831BFCC23C2}">
-  <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55BEB37B-B28E-4F60-BECB-CD35E74B4C36}">
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="30" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1409,59 +1369,114 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>108</v>
+        <v>11</v>
       </c>
       <c r="C2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>109</v>
+        <v>12</v>
       </c>
       <c r="C3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>111</v>
+        <v>13</v>
       </c>
       <c r="C4" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>113</v>
-      </c>
-      <c r="C5">
-        <v>1234</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>28</v>
+        <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>114</v>
-      </c>
-      <c r="C6">
-        <v>330</v>
+        <v>48</v>
+      </c>
+      <c r="C6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
+        <v>49</v>
+      </c>
+      <c r="C10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C11" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -1470,15 +1485,15 @@
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDDAC24B-DC90-49E6-BD31-6F210026CA6D}">
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82865F4C-F847-4F90-8B11-C831BFCC23C2}">
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="25.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1489,37 +1504,59 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>115</v>
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>108</v>
       </c>
       <c r="C2" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>116</v>
+        <v>5</v>
+      </c>
+      <c r="B3" t="s">
+        <v>109</v>
       </c>
       <c r="C3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>117</v>
+        <v>5</v>
+      </c>
+      <c r="B4" t="s">
+        <v>111</v>
       </c>
       <c r="C4" t="s">
-        <v>51</v>
+        <v>112</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" t="s">
+        <v>113</v>
+      </c>
+      <c r="C5">
+        <v>1234</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" t="s">
+        <v>114</v>
+      </c>
+      <c r="C6">
+        <v>330</v>
       </c>
     </row>
   </sheetData>
@@ -1528,15 +1565,15 @@
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6F7845C-214C-4C02-A5F4-6F38FB46E35D}">
-  <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDDAC24B-DC90-49E6-BD31-6F210026CA6D}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="33.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="41.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1547,81 +1584,37 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>118</v>
-      </c>
-      <c r="C2">
-        <v>365</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>3</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="C2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" t="s">
-        <v>119</v>
-      </c>
-      <c r="C3">
-        <v>455</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+        <v>3</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="C3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" t="s">
-        <v>52</v>
+        <v>3</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>117</v>
       </c>
       <c r="C4" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" t="s">
-        <v>54</v>
-      </c>
-      <c r="C5" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>5</v>
-      </c>
-      <c r="B6" t="s">
-        <v>55</v>
-      </c>
-      <c r="C6" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>5</v>
-      </c>
-      <c r="B7" t="s">
-        <v>57</v>
-      </c>
-      <c r="C7" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B8" t="s">
-        <v>59</v>
-      </c>
-      <c r="C8" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -1630,15 +1623,117 @@
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6F7845C-214C-4C02-A5F4-6F38FB46E35D}">
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="33.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41.1796875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>118</v>
+      </c>
+      <c r="C2">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" t="s">
+        <v>119</v>
+      </c>
+      <c r="C3">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C4" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" t="s">
+        <v>54</v>
+      </c>
+      <c r="C5" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>55</v>
+      </c>
+      <c r="C6" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" t="s">
+        <v>57</v>
+      </c>
+      <c r="C7" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" t="s">
+        <v>59</v>
+      </c>
+      <c r="C8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE64D93B-66B6-48F6-99BC-E4BA23590E06}">
   <dimension ref="A1:C10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="23" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1649,7 +1744,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -1660,7 +1755,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -1671,7 +1766,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -1682,7 +1777,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -1693,7 +1788,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
@@ -1704,7 +1799,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>3</v>
       </c>
@@ -1715,7 +1810,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>3</v>
       </c>
@@ -1726,7 +1821,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>3</v>
       </c>
@@ -1737,7 +1832,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>3</v>
       </c>
@@ -1754,15 +1849,107 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D9414A1A-FB8B-4B66-A538-3949CB53646C}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="7.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.36328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C2" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>63</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>64</v>
+      </c>
+      <c r="C5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>65</v>
+      </c>
+      <c r="C6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>66</v>
+      </c>
+      <c r="C7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E83D430-2DDF-4C96-A733-8F6A18593E6C}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="30.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1773,7 +1960,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1784,7 +1971,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1795,7 +1982,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1806,7 +1993,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1817,7 +2004,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -1828,7 +2015,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -1845,16 +2032,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D03E8B95-40CB-49F7-AF29-3A2B27B21A61}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="19.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1865,7 +2052,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1876,7 +2063,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1887,7 +2074,7 @@
         <v>1825</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1898,7 +2085,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1907,49 +2094,6 @@
       </c>
       <c r="C5" t="s">
         <v>73</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C485CB82-74B9-4E1E-9CE3-715999920922}">
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="C2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="C3">
-        <v>1825</v>
       </c>
     </row>
   </sheetData>
@@ -1958,15 +2102,58 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C485CB82-74B9-4E1E-9CE3-715999920922}">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C3">
+        <v>1825</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F19EA7F8-0885-4456-A6E5-96AB05BF51FA}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="25.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="40.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1977,7 +2164,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1988,7 +2175,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1999,7 +2186,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -2016,17 +2203,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C0E25E5-8973-4E31-A3CE-0B2930FA70C8}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="40.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2037,7 +2224,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2048,7 +2235,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -2057,152 +2244,6 @@
       </c>
       <c r="C3" t="s">
         <v>10</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B47C19A-7081-4532-8CD1-2D1BC531686A}">
-  <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="2" max="2" width="27.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.77734375" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="C2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="C3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="C4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="C5" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="C6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="C7" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="C8" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="C9" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="C10" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="C11" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>3</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="C12" t="s">
-        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -2211,15 +2252,15 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4BADE6FB-E965-4263-BE22-5F02F8843366}">
-  <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B47C19A-7081-4532-8CD1-2D1BC531686A}">
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="27" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="40.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2230,81 +2271,125 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>16</v>
+        <v>3</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>78</v>
       </c>
       <c r="C2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" t="s">
-        <v>17</v>
+        <v>3</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>79</v>
       </c>
       <c r="C3" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" t="s">
-        <v>67</v>
-      </c>
-      <c r="C4">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+        <v>3</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="C4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C5">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+        <v>3</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="C5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>19</v>
-      </c>
-      <c r="B6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C6">
-        <v>10000</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+        <v>3</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="C6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>19</v>
-      </c>
-      <c r="B7" t="s">
-        <v>22</v>
-      </c>
-      <c r="C7">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+        <v>3</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="C7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>19</v>
-      </c>
-      <c r="B8" t="s">
-        <v>23</v>
-      </c>
-      <c r="C8">
-        <v>10000</v>
+        <v>3</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="C8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="C9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="C10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="C11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="C12" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -2313,15 +2398,15 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{531E32A4-7E13-4409-95B5-698B0506DEBB}">
-  <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4BADE6FB-E965-4263-BE22-5F02F8843366}">
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="26.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2332,70 +2417,81 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="C2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="C3" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>28</v>
+        <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>29</v>
-      </c>
-      <c r="C4" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+        <v>67</v>
+      </c>
+      <c r="C4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="B5" t="s">
-        <v>32</v>
-      </c>
-      <c r="C5" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+        <v>20</v>
+      </c>
+      <c r="C5">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="B6" t="s">
-        <v>34</v>
-      </c>
-      <c r="C6" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+        <v>21</v>
+      </c>
+      <c r="C6">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="B7" t="s">
-        <v>35</v>
-      </c>
-      <c r="C7" t="s">
-        <v>33</v>
+        <v>22</v>
+      </c>
+      <c r="C7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8">
+        <v>10000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added Sanity Test Cases in Modules and added files Collab, Dynamic Form, Send Email, Side Bar
</commit_message>
<xml_diff>
--- a/src/main/resources/Program_Field_Values_QA_org.xlsx
+++ b/src/main/resources/Program_Field_Values_QA_org.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27126"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27231"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F81410B6-FA6A-4A0B-9175-56762F212B7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FC43C5C-484F-4D34-8733-10F70DF1209C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="10" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="15" activeTab="19" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="StaticRecordProgramCreation" sheetId="39" r:id="rId1"/>
@@ -27,6 +27,7 @@
     <sheet name="SiteVisitCreation_v" sheetId="34" r:id="rId17"/>
     <sheet name="SiteVisitEdition_v" sheetId="35" r:id="rId18"/>
     <sheet name="GeneralReviewForm_v" sheetId="36" r:id="rId19"/>
+    <sheet name="Contacts" sheetId="41" r:id="rId20"/>
   </sheets>
   <calcPr calcId="179017"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="373" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="385" uniqueCount="140">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -440,6 +441,24 @@
   </si>
   <si>
     <t>Automation Program For Announcement</t>
+  </si>
+  <si>
+    <t>fieldFirstName</t>
+  </si>
+  <si>
+    <t>Thor</t>
+  </si>
+  <si>
+    <t>fieldLastName</t>
+  </si>
+  <si>
+    <t>America</t>
+  </si>
+  <si>
+    <t>fieldProjectRole__c</t>
+  </si>
+  <si>
+    <t>Program Manager</t>
   </si>
 </sst>
 </file>
@@ -1927,6 +1946,94 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CCC7C533-9694-4FF8-A93E-689ECBD164CC}">
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="23" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="1"/>
+      <c r="B7" s="1"/>
+      <c r="C7" s="1"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="1"/>
+      <c r="B8" s="1"/>
+      <c r="C8" s="1"/>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="1"/>
+      <c r="B9" s="1"/>
+      <c r="C9" s="1"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="1"/>
+      <c r="B10" s="1"/>
+      <c r="C10" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E83D430-2DDF-4C96-A733-8F6A18593E6C}">
   <dimension ref="A1:C7"/>

</xml_diff>